<commit_message>
- fix param in action - fix query for calibration due job - formatted columns as Date in Excel files
</commit_message>
<xml_diff>
--- a/api/templates/device_calibration_report/uk.xlsx
+++ b/api/templates/device_calibration_report/uk.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\device_calibration_report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-4\api\templates\device_calibration_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB1D520B-D518-4A95-92B2-F99DBFC8569D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Калібрування пристрою" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -83,7 +82,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -175,16 +177,38 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -193,7 +217,12 @@
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+      <tableStyleElement type="wholeTable" dxfId="1"/>
+      <tableStyleElement type="headerRow" dxfId="0"/>
+    </tableStyle>
+  </tableStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -569,7 +598,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E501"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -630,13 +659,13 @@
       <c r="B8" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="9" t="str">
+      <c r="E8" s="8" t="str">
         <f ca="1">IF(ISNUMBER(D8),IF(D8-TODAY()&lt;0,"OVERDUE",INT(D8-TODAY())),"")</f>
         <v/>
       </c>
@@ -2615,7 +2644,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A8:E100000">
-    <cfRule type="expression" dxfId="0" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>IF(ISNUMBER($D8),$D8-TODAY()&lt;0,0)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>